<commit_message>
Simplify the cost bar to two segments for the slide
Split into lab analysis, refills and subscription, the second bar was three
bands of which two were small — detail that does not survive being read from
the back of a room.

Now two: lab analysis and Fluorsight. That keeps the one thing the split was
actually there for, which is that half the remaining spend is still the
laboratory, so nobody reads the second bar as our invoice. £25,000 plus
£25,000, summing to the £50,000 in the title. The full breakdown stays in the
table directly above the chart data.

Also ignores Excel's ~$ lock files.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcpMcZ5nmubFgAzx2U2w1E
</commit_message>
<xml_diff>
--- a/docs/fluorsight-model.xlsx
+++ b/docs/fluorsight-model.xlsx
@@ -309,34 +309,6 @@
           <val>
             <numRef>
               <f>'Model'!$C$30:$C$31</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'Model'!D29</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1BAF7A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Model'!$A$30:$A$31</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Model'!$D$30:$D$31</f>
             </numRef>
           </val>
         </ser>
@@ -3319,12 +3291,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Refills</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Subscription</t>
+          <t>Fluorsight</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3306,6 @@
         <v/>
       </c>
       <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3352,12 +3318,13 @@
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>B9</f>
-        <v/>
-      </c>
-      <c r="D31" s="10">
-        <f>B10</f>
-        <v/>
+        <f>B9+B10</f>
+        <v/>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Fluorsight = refills + subscription. The device is a one-off and is excluded from an annual-cost bar.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extend the escalation sensitivity to 95%, and correct what it claims
Table A ran 5-55%, which never reached the point where the model fails.
Extended to 95% it does: the saving crosses zero at about 80% escalation.
That is a second break-even and worth having — if the screen sends four in
five samples to the lab anyway, triage has added cost for nothing.

Two things that had to change with it. The chart was titled "the saving holds
across the rate we are least sure of", which the new range makes false, so it
now reads "Triage pays until about 80% of screened samples escalate". And the
category axis was rendering 0.05, 0.1, 0.15 because only the cells carried a
percent format, not the axis.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcpMcZ5nmubFgAzx2U2w1E
</commit_message>
<xml_diff>
--- a/docs/fluorsight-model.xlsx
+++ b/docs/fluorsight-model.xlsx
@@ -506,7 +506,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>The saving holds across the rate we are least sure of</a:t>
+              <a:t>Triage pays until about 80% of screened samples escalate</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -541,12 +541,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Sensitivity'!$A$6:$A$16</f>
+              <f>'Sensitivity'!$A$6:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Sensitivity'!$C$6:$C$16</f>
+              <f>'Sensitivity'!$C$6:$C$24</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -582,7 +582,7 @@
           </tx>
           <overlay val="0"/>
         </title>
-        <numFmt formatCode="General" sourceLinked="0"/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <spPr>
@@ -3338,7 +3338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3887,6 +3887,17 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" s="20" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="B17" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A17,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C17" s="17">
+        <f>B17/Model!$B$6</f>
+        <v/>
+      </c>
       <c r="E17" s="10" t="n">
         <v>300</v>
       </c>
@@ -3896,6 +3907,17 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" s="20" t="n">
+        <v>0.6500000000000001</v>
+      </c>
+      <c r="B18" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A18,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
+        <f>B18/Model!$B$6</f>
+        <v/>
+      </c>
       <c r="E18" s="10" t="n">
         <v>325</v>
       </c>
@@ -3905,6 +3927,17 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" s="20" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="B19" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A19,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C19" s="17">
+        <f>B19/Model!$B$6</f>
+        <v/>
+      </c>
       <c r="E19" s="10" t="n">
         <v>350</v>
       </c>
@@ -3914,6 +3947,17 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" s="20" t="n">
+        <v>0.7500000000000001</v>
+      </c>
+      <c r="B20" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A20,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
+        <f>B20/Model!$B$6</f>
+        <v/>
+      </c>
       <c r="E20" s="10" t="n">
         <v>375</v>
       </c>
@@ -3923,11 +3967,61 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" s="20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B21" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A21,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C21" s="17">
+        <f>B21/Model!$B$6</f>
+        <v/>
+      </c>
       <c r="E21" s="10" t="n">
         <v>400</v>
       </c>
       <c r="F21" s="10">
         <f>Assumptions!$B$6*E21-(ROUND(Assumptions!$B$6*Assumptions!$B$7,0)*E21+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="B22" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A22,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C22" s="17">
+        <f>B22/Model!$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="n">
+        <v>0.9000000000000001</v>
+      </c>
+      <c r="B23" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A23,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C23" s="17">
+        <f>B23/Model!$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="B24" s="10">
+        <f>Model!$B$6-(ROUND(Assumptions!$B$6*A24,0)*Assumptions!$B$8+Model!$B$9+Model!$B$10+Model!$B$11)</f>
+        <v/>
+      </c>
+      <c r="C24" s="17">
+        <f>B24/Model!$B$6</f>
         <v/>
       </c>
     </row>

</xml_diff>